<commit_message>
BDOI-template FRS packs: verification fixes
- Workbooks recalculated in LibreOffice: no formula errors; very wide sheets print on A3 landscape
- BRD-06: the note of Annex AN.3 before its table (no page with the note alone)
- BRD-11 and others: a tall figure with a How to read it note shrinks so the note stays on its page
- Headings 1 and 2 in BDOI's title case; double spaces across runs removed; 'renewal renewal' fixed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Effort_Estimate_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Effort_Estimate_v1.0.xlsx
@@ -3867,7 +3867,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;8 &amp;K004EA8CR Effort Estimate&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
@@ -4190,7 +4190,7 @@
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;8 &amp;K004EA8CR Effort Estimate&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
@@ -4351,7 +4351,7 @@
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;8 &amp;K004EA8CR Effort Estimate&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
@@ -5423,7 +5423,7 @@
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;8 &amp;K004EA8CR Effort Estimate&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>

</xml_diff>